<commit_message>
Atualiza a estrutura dos indicadores para incluir espaços e filtrar apenas os indicadores disponíveis; salva as variáveis atualizadas no arquivo indicadores.csv.
</commit_message>
<xml_diff>
--- a/ods/db/resultados/Objetivo7.xlsx
+++ b/ods/db/resultados/Objetivo7.xlsx
@@ -4,14 +4,11 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Indicador 7.1.1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Indicador 7.1.2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Indicador 7.2.1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Indicador 7.3.1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Indicador 7.b.1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8799,1489 +8796,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID_INDICADOR</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CODG_UND_MED</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>VLR_VAR</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>CODG_UND_FED</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>DESC_UND_FED</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>CODG_VAR</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>CODG_ANO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>43.6</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>41.9</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>40.6</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>39.7</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>41.5</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>43.7</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>43.4</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>45.8</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>46.4</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>48.7</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>45.0</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Indicador  7.2.1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>47.4</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>9340</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID_INDICADOR</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CODG_UND_MED</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>VLR_VAR</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>CODG_UND_FED</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>DESC_UND_FED</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>CODG_VAR</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>CODG_ANO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>0.090</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0.092</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>0.093</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>0.096</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0.098</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0.097</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>0.098</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>0.095</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>0.095</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>0.096</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>0.096</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Indicador  7.3.1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1724</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>0.093</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>9338</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID_INDICADOR</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CODG_UND_MED</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>VLR_VAR</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>CODG_UND_FED</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>DESC_UND_FED</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>CODG_VAR</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>CODG_ANO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>470.54</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2011</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>482.59</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2012</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>496.99</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2013</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>525.36</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2014</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>551.00</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>588.85</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>617.59</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2017</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>648.68</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>682.83</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>704.62</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>745.58</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Indicador  7.b.1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1751</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>810.73</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>10527</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>